<commit_message>
i added results for third term exams
</commit_message>
<xml_diff>
--- a/Master/2025_and_2026/JSS2.xlsx
+++ b/Master/2025_and_2026/JSS2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Reporter\Master\2025_and_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2FF7DE-0500-4C8E-B5AA-791F14C94958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A233557-50CA-4D44-9B39-30848887B765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{238F1817-8B51-4C71-B722-8E62592C6D1C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="91">
   <si>
     <t>English Studies</t>
   </si>
@@ -78,9 +78,6 @@
     <t>j23.jpg</t>
   </si>
   <si>
-    <t>j25.jpg</t>
-  </si>
-  <si>
     <t>Four</t>
   </si>
   <si>
@@ -295,6 +292,12 @@
   </si>
   <si>
     <t>Mujeeb</t>
+  </si>
+  <si>
+    <t>Ishola</t>
+  </si>
+  <si>
+    <t>mujeeb.jpg</t>
   </si>
 </sst>
 </file>
@@ -710,79 +713,79 @@
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>36</v>
       </c>
-      <c r="F1" t="s">
-        <v>37</v>
-      </c>
       <c r="G1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I1" t="s">
         <v>43</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>44</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>45</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" t="s">
         <v>46</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>50</v>
       </c>
-      <c r="M1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>51</v>
       </c>
-      <c r="O1" t="s">
-        <v>52</v>
-      </c>
       <c r="P1" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q1" t="s">
         <v>78</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>79</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>80</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>81</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>82</v>
-      </c>
-      <c r="U1" t="s">
-        <v>83</v>
       </c>
       <c r="V1" t="s">
         <v>0</v>
       </c>
       <c r="W1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="X1" t="s">
         <v>1</v>
       </c>
       <c r="Y1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="Z1" t="s">
         <v>2</v>
@@ -797,7 +800,7 @@
         <v>5</v>
       </c>
       <c r="AD1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AE1" t="s">
         <v>6</v>
@@ -806,7 +809,7 @@
         <v>7</v>
       </c>
       <c r="AG1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.35">
@@ -817,10 +820,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
@@ -829,31 +832,31 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" t="s">
         <v>54</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>55</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>56</v>
-      </c>
-      <c r="L2" t="s">
-        <v>57</v>
       </c>
       <c r="M2" s="5">
         <v>37904</v>
       </c>
       <c r="N2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="O2" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>59</v>
       </c>
       <c r="P2">
         <v>1</v>
@@ -915,10 +918,10 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
         <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
@@ -927,31 +930,31 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" t="s">
         <v>60</v>
-      </c>
-      <c r="J3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K3" t="s">
-        <v>56</v>
-      </c>
-      <c r="L3" t="s">
-        <v>61</v>
       </c>
       <c r="M3" s="5">
         <v>37691</v>
       </c>
       <c r="N3" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="O3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="P3">
         <v>1</v>
@@ -1013,10 +1016,10 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -1025,31 +1028,31 @@
         <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" t="s">
         <v>48</v>
       </c>
-      <c r="J4" t="s">
-        <v>49</v>
-      </c>
       <c r="K4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M4" s="5">
         <v>37967</v>
       </c>
       <c r="N4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="O4" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="P4">
         <v>1</v>
@@ -1111,10 +1114,10 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -1123,31 +1126,31 @@
         <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" t="s">
+        <v>55</v>
+      </c>
+      <c r="L5" t="s">
         <v>67</v>
-      </c>
-      <c r="J5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" t="s">
-        <v>56</v>
-      </c>
-      <c r="L5" t="s">
-        <v>68</v>
       </c>
       <c r="M5" s="5">
         <v>37665</v>
       </c>
       <c r="N5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="O5" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="P5">
         <v>1</v>
@@ -1209,43 +1212,43 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" t="s">
         <v>88</v>
       </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>89</v>
-      </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>90</v>
       </c>
       <c r="G6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" t="s">
         <v>48</v>
       </c>
-      <c r="J6" t="s">
-        <v>49</v>
-      </c>
       <c r="K6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M6" s="5">
         <v>37755</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="P6">
         <v>1</v>
@@ -1277,7 +1280,7 @@
       <c r="Y6">
         <v>1</v>
       </c>
-      <c r="AA6">
+      <c r="Z6">
         <v>1</v>
       </c>
       <c r="AB6">
@@ -1307,43 +1310,43 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" t="s">
-        <v>19</v>
-      </c>
       <c r="G7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" t="s">
         <v>48</v>
       </c>
-      <c r="J7" t="s">
-        <v>49</v>
-      </c>
       <c r="K7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M7" s="5">
         <v>37636</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P7">
         <v>1</v>
@@ -1405,43 +1408,43 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
       <c r="G8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J8" t="s">
         <v>48</v>
       </c>
-      <c r="J8" t="s">
-        <v>49</v>
-      </c>
       <c r="K8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M8" s="5">
         <v>37880</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P8">
         <v>1</v>
@@ -1503,43 +1506,43 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
         <v>22</v>
       </c>
-      <c r="F9" t="s">
-        <v>23</v>
-      </c>
       <c r="G9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" t="s">
         <v>48</v>
       </c>
-      <c r="J9" t="s">
-        <v>49</v>
-      </c>
       <c r="K9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M9" s="5">
         <v>37850</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P9">
         <v>1</v>

</xml_diff>